<commit_message>
Add social media preview, simplify match rows to flags-only, and improve ranking-based simulation
</commit_message>
<xml_diff>
--- a/third-place-matchups.xlsx
+++ b/third-place-matchups.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rredondo/Desktop/world-cup-simulator/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{634B7824-2A4B-AB4B-8740-C6C69DD39A4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C8F07E1-0F93-F748-A7A4-EAC753B02F2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="33600" yWindow="-3200" windowWidth="38400" windowHeight="21000" xr2:uid="{4C310F0F-A4CF-B546-BAE6-266BCDEBA1B7}"/>
+    <workbookView xWindow="44380" yWindow="240" windowWidth="33600" windowHeight="18940" xr2:uid="{4C310F0F-A4CF-B546-BAE6-266BCDEBA1B7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7954" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7954" uniqueCount="35">
   <si>
     <t>E</t>
   </si>
@@ -160,6 +160,9 @@
   </si>
   <si>
     <t>Concat</t>
+  </si>
+  <si>
+    <t></t>
   </si>
 </sst>
 </file>
@@ -18727,7 +18730,7 @@
         <v>100001111111</v>
       </c>
       <c r="AA167" s="2" t="s">
-        <v>16</v>
+        <v>34</v>
       </c>
       <c r="AB167" s="2" t="s">
         <v>13</v>

</xml_diff>